<commit_message>
refactor: rename exam HTML files to examwords- prefix and update links in index, README, and Excel
</commit_message>
<xml_diff>
--- a/2026_段考國注百題卷_網址總覽表.xlsx
+++ b/2026_段考國注百題卷_網址總覽表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\2026_段考國注百字卷\上傳github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AC174A6-F1D9-4115-ACCE-FCC3C466D1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2626A879-B496-49EA-9B82-5061167386F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{87A84288-BF2B-4898-A379-4277A2B4626E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4135F7E8-3851-46A8-ADF6-B199A7862A82}"/>
   </bookViews>
   <sheets>
     <sheet name="段考國注百題卷網址總覽" sheetId="1" r:id="rId1"/>
@@ -104,13 +104,13 @@
     <t>7-1-1七上段一國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-7-1-1.html</t>
+    <t>examwords-7-1-1.html</t>
   </si>
   <si>
     <t>第一課、第三課、自學一（含語文常識一）</t>
   </si>
   <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-7-1-1.html</t>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-7-1-1.html</t>
   </si>
   <si>
     <t>閃卡翻面記憶、百題大卷測驗/講義、錯題本專區、星號收藏</t>
@@ -122,13 +122,13 @@
     <t>7-1-2七上段二國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-7-1-2.html</t>
+    <t>examwords-7-1-2.html</t>
   </si>
   <si>
     <t>第四課～第六課（含語文常識二）</t>
   </si>
   <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-7-1-2.html</t>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-7-1-2.html</t>
   </si>
   <si>
     <t>第三次段考</t>
@@ -137,13 +137,13 @@
     <t>7-1-3七上段三國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-7-1-3.html</t>
+    <t>examwords-7-1-3.html</t>
   </si>
   <si>
     <t>第七課～第九課</t>
   </si>
   <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-7-1-3.html</t>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-7-1-3.html</t>
   </si>
   <si>
     <t>七年級下學期</t>
@@ -152,34 +152,34 @@
     <t>7-2-1七下段一國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-7-2-1.html</t>
+    <t>examwords-7-2-1.html</t>
   </si>
   <si>
     <t>第一課、第三課、自學一</t>
   </si>
   <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-7-2-1.html</t>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-7-2-1.html</t>
   </si>
   <si>
     <t>7-2-2七下段二國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-7-2-2.html</t>
+    <t>examwords-7-2-2.html</t>
   </si>
   <si>
     <t>第四課～第六課</t>
   </si>
   <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-7-2-2.html</t>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-7-2-2.html</t>
   </si>
   <si>
     <t>7-2-3七下段三國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-7-2-3.html</t>
-  </si>
-  <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-7-2-3.html</t>
+    <t>examwords-7-2-3.html</t>
+  </si>
+  <si>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-7-2-3.html</t>
   </si>
   <si>
     <t>八年級上學期</t>
@@ -188,13 +188,13 @@
     <t>8-1-1八上段一國注百題[練習神器].html</t>
   </si>
   <si>
-    <t>exam-8-1-1.html</t>
+    <t>examwords-8-1-1.html</t>
   </si>
   <si>
     <t>第一課～第三課（含語文常識一）</t>
   </si>
   <si>
-    <t>https://oaoadna-1313.github.io/2026_exam100words/exam-8-1-1.html</t>
+    <t>https://oaoadna-1313.github.io/2026_exam100words/examwords-8-1-1.html</t>
   </si>
 </sst>
 </file>
@@ -713,7 +713,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{630320C5-BEDB-4B53-AC21-F35F9A666DFB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472688B7-573D-4C19-9E5A-5EDF70AABD26}">
   <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
@@ -721,10 +721,10 @@
     <col min="2" max="2" width="14.6328125" customWidth="1"/>
     <col min="3" max="3" width="13.6328125" customWidth="1"/>
     <col min="4" max="4" width="36.6328125" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" customWidth="1"/>
+    <col min="5" max="5" width="24.6328125" customWidth="1"/>
     <col min="6" max="6" width="35.6328125" customWidth="1"/>
     <col min="7" max="7" width="8.6328125" customWidth="1"/>
-    <col min="8" max="8" width="58.6328125" customWidth="1"/>
+    <col min="8" max="8" width="64.6328125" customWidth="1"/>
     <col min="9" max="9" width="46.6328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1022,14 +1022,14 @@
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="H4" r:id="rId1" tooltip="https://oaoadna-1313.github.io/2026_exam100words/index.html" xr:uid="{E0FF1711-2AFD-469A-8148-0C2E1B6F4371}"/>
-    <hyperlink ref="H5" r:id="rId2" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-7-1-1.html" xr:uid="{8BAFD15E-FF39-466A-B72D-6AECE3BC5F03}"/>
-    <hyperlink ref="H6" r:id="rId3" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-7-1-2.html" xr:uid="{389291AC-2A39-475B-A640-5791211AA555}"/>
-    <hyperlink ref="H7" r:id="rId4" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-7-1-3.html" xr:uid="{60FFCFA5-3515-4033-8BAA-1F119BAE5EA8}"/>
-    <hyperlink ref="H8" r:id="rId5" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-7-2-1.html" xr:uid="{8853A501-F807-4E05-B4F2-40196F8305BE}"/>
-    <hyperlink ref="H9" r:id="rId6" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-7-2-2.html" xr:uid="{751895A4-E40D-43F5-97FC-92BE18BB4D8D}"/>
-    <hyperlink ref="H10" r:id="rId7" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-7-2-3.html" xr:uid="{09C96600-78DD-406A-8BC2-32034A7D7F57}"/>
-    <hyperlink ref="H11" r:id="rId8" tooltip="https://oaoadna-1313.github.io/2026_exam100words/exam-8-1-1.html" xr:uid="{353CDA1F-4839-4042-B2BA-AF8CCB8E5A45}"/>
+    <hyperlink ref="H4" r:id="rId1" tooltip="https://oaoadna-1313.github.io/2026_exam100words/index.html" xr:uid="{AB90FC3A-92F6-4E94-AD40-68670E989BF8}"/>
+    <hyperlink ref="H5" r:id="rId2" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-7-1-1.html" xr:uid="{C283D1C4-795B-4978-AE1A-B3ECDBF5C733}"/>
+    <hyperlink ref="H6" r:id="rId3" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-7-1-2.html" xr:uid="{8E50E909-65E3-4FA1-9361-EB8D35703A7F}"/>
+    <hyperlink ref="H7" r:id="rId4" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-7-1-3.html" xr:uid="{2FF1E5EC-FE6C-439B-9C80-DAC462EDD462}"/>
+    <hyperlink ref="H8" r:id="rId5" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-7-2-1.html" xr:uid="{2EBD571A-7424-4D5A-AF07-E08E05C7EE72}"/>
+    <hyperlink ref="H9" r:id="rId6" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-7-2-2.html" xr:uid="{1289F404-7DEE-4004-93BA-B970B4022B32}"/>
+    <hyperlink ref="H10" r:id="rId7" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-7-2-3.html" xr:uid="{D30A1A66-D263-4A7F-BCAB-72806344CAE3}"/>
+    <hyperlink ref="H11" r:id="rId8" tooltip="https://oaoadna-1313.github.io/2026_exam100words/examwords-8-1-1.html" xr:uid="{18423637-C927-46BB-AABC-ED24E3A1DF97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>